<commit_message>
build: update data generation script and bump version to 1.2.0
Refactor the `generate-data-xlsx.mjs` script to use `exceljs` instead of manual XML string construction. This ensures that embedded images (like the logo) are preserved correctly when the Excel file is edited and re-saved.

- Add `exceljs` dependency
- Update version to 1.2.0 in `package.json`, `app-info.ts`, and `generate-data-xlsx.mjs`
- Update release notes to reflect dark mode support
- Update `data.xlsx` with new version and notes
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,15 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
-  <workbookPr/>
-  <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Data"/>
+    <sheet sheetId="1" name="Data" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -25,14 +22,15 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.1.0</t>
+    <t>1.2.0</t>
   </si>
   <si>
     <t>Version-Release-Update</t>
   </si>
   <si>
-    <t>Version 1.1.0
-- Drag &amp; drop: drop .docx labels or .zip archives anywhere in Check &amp; fix to scan them.</t>
+    <t xml:space="preserve">Version 1.2.0
+- Drag &amp; drop: drop .docx labels or .zip archives anywhere in Check &amp; fix to scan them.
+- Dark mode: follows your system theme by default; switch anytime with the sun/moon button in the top bar.</t>
   </si>
   <si>
     <t>Logo</t>
@@ -50,28 +48,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF17211f"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -82,14 +69,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -101,44 +81,71 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>31000</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>24999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1524000" cy="552450"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -146,10 +153,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -158,7 +165,7 @@
         <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F818D"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="C0504D"/>
@@ -187,71 +194,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -275,53 +282,50 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="9500"/>
+              <a:shade val="95000"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -331,7 +335,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -340,7 +344,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -349,7 +353,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -357,10 +361,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -389,7 +393,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="20000"/>
+                <a:shade val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -402,12 +406,13 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
+                <a:shade val="30000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -419,64 +424,102 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" style="7" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="62.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="90" customFormat="1" s="5">
-      <c r="A3" s="4" t="s">
+    <row r="3" ht="62" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18" customFormat="1" s="5">
-      <c r="A4" s="4" t="s">
+    <row r="4" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18" customFormat="1" s="5">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ui): implement full-size PDF label preview
Introduces a new PDF-based preview system for label creation, replacing
the previous image-based barcode preview. This provides a more accurate
representation of the final printed label.

- Add `pdfjs-dist` and `pdf-lib` dependencies for PDF rendering.
- Implement `LabelPdfPreview` component using `pdf.js` to render a
  server-side generated PDF onto a canvas.
- Refactor label geometry into a dedicated `label-geometry.ts` module.
- Update `docx-writer` to optimize ingredient text placement, ensuring
  content starts immediately after the "Ingredients:" label to prevent
  unnecessary line wraps.
- Adjust label layout to provide more vertical space for ingredients.
- Update version to 1.2.1 and refresh release notes.

Ref: Issue/problems-to-fix.md
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -22,15 +22,15 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.0</t>
+    <t>1.2.1</t>
   </si>
   <si>
     <t>Version-Release-Update</t>
   </si>
   <si>
-    <t xml:space="preserve">Version 1.2.0
-- Drag &amp; drop: drop .docx labels or .zip archives anywhere in Check &amp; fix to scan them.
-- Dark mode: follows your system theme by default; switch anytime with the sun/moon button in the top bar.</t>
+    <t xml:space="preserve">Version 1.2.1
+- Label layout: more room for ingredients; the list starts right after "Ingredients:".
+- Create preview: full-size PDF preview that matches the printed label.</t>
   </si>
   <si>
     <t>Logo</t>

</xml_diff>

<commit_message>
fix(domain): prevent mid-word line breaking in prose text boxes
Implements whole-word wrapping for product name, storage instructions,
and ingredients text boxes in the DOCX generator. This prevents
Latin words from being split at the right edge of the box due to
the template's East Asian layout compatibility rules.

The barcode number box remains character-breakable to allow long
GS1 numbers to wrap if necessary.

- Update version to 1.2.2
- Add `wrapWholeWords` utility to `docx-writer.ts`
- Add regression tests for word-wrap behavior in `docx-writer.test.ts`
- Update documentation in `agents.md` regarding versioning and data
  generation workflow
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -22,15 +22,14 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.1</t>
+    <t>1.2.2</t>
   </si>
   <si>
     <t>Version-Release-Update</t>
   </si>
   <si>
-    <t xml:space="preserve">Version 1.2.1
-- Label layout: more room for ingredients; the list starts right after "Ingredients:".
-- Create preview: full-size PDF preview that matches the printed label.</t>
+    <t xml:space="preserve">v1.2.2
+- Word breaking fix</t>
   </si>
   <si>
     <t>Logo</t>

</xml_diff>

<commit_message>
chore(config): bump version to 1.2.3 and update release notes
Update the application version and release update text to reflect
recent improvements to label typography and word wrapping behavior.

- Increment version from 1.2.2 to 1.2.3
- Update `DEFAULT_APP_INFO` with detailed release notes
- Update `generate-data-xlsx.mjs` script to use new version and notes
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -22,14 +22,15 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.2</t>
+    <t>1.2.3</t>
   </si>
   <si>
     <t>Version-Release-Update</t>
   </si>
   <si>
-    <t xml:space="preserve">v1.2.2
-- Word breaking fix</t>
+    <t xml:space="preserve">v1.2.3
+- Words no longer split across lines on labels.
+- Ingredient text stays larger and fills the label box better.</t>
   </si>
   <si>
     <t>Logo</t>

</xml_diff>